<commit_message>
[0.1.2] - 2025-10-24 Added remote camera exposure, color, and focus control
</commit_message>
<xml_diff>
--- a/PTZ/Action_Item_List.xlsx
+++ b/PTZ/Action_Item_List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/99d2d0efc5e421e1/Working_Files/CPC_Production/PTZ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_F25DC773A252ABDACC1048B0395B70645BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA747CCD-E9A1-4EA6-8CFA-A9FE8752FF86}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="11_F25DC773A252ABDACC1048B0395B70645BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43FC79B8-93E0-4758-A0DB-76E5A4784B8D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
   <si>
     <t>What</t>
   </si>
@@ -49,6 +49,12 @@
   </si>
   <si>
     <t>Camera Exposure and Color Balance</t>
+  </si>
+  <si>
+    <t>Steve &amp; Mike</t>
+  </si>
+  <si>
+    <t>Monitor 10/24/25</t>
   </si>
 </sst>
 </file>
@@ -84,8 +90,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -101,6 +108,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -396,15 +407,42 @@
       <c r="A2" t="s">
         <v>7</v>
       </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1">
+        <v>45951</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1">
+        <v>45951</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1">
+        <v>45951</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>